<commit_message>
correct the math flow for ampseq
</commit_message>
<xml_diff>
--- a/inst/extdata/makers_details.xlsx
+++ b/inst/extdata/makers_details.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/24b25e554f22146a/Masters Class notes/AIMS Rwanda/Thesis Phase/Publication Phase/Refactoring MalReBay/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dev\MalReBay-Package\MalReBay\inst\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{D403CC85-76BC-4478-A233-D1D2E70AF80F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{26417E7E-DC63-4EC6-BCA3-4C1AF67F6512}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F742158D-9736-4AE3-A469-7175A3109C10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B200665-48F8-48D7-B17C-7D3B5710279D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="62">
   <si>
     <t>marker_id</t>
   </si>
@@ -168,6 +168,60 @@
   </si>
   <si>
     <t>TRAP3</t>
+  </si>
+  <si>
+    <t>cpmp1</t>
+  </si>
+  <si>
+    <t>celtos</t>
+  </si>
+  <si>
+    <t>surfin1.1</t>
+  </si>
+  <si>
+    <t>ama1-D2</t>
+  </si>
+  <si>
+    <t>ama1-D2.1</t>
+  </si>
+  <si>
+    <t>TRAP2</t>
+  </si>
+  <si>
+    <t>ama1-D3.3</t>
+  </si>
+  <si>
+    <t>csp1</t>
+  </si>
+  <si>
+    <t>msp7.2</t>
+  </si>
+  <si>
+    <t>ama1-D2.3</t>
+  </si>
+  <si>
+    <t>ama1-D3.2</t>
+  </si>
+  <si>
+    <t>cpp3</t>
+  </si>
+  <si>
+    <t>msp7.3</t>
+  </si>
+  <si>
+    <t>cpmp3</t>
+  </si>
+  <si>
+    <t>TRAP4_</t>
+  </si>
+  <si>
+    <t>ama1-D3.4</t>
+  </si>
+  <si>
+    <t>cpmp2</t>
+  </si>
+  <si>
+    <t>cpp1</t>
   </si>
 </sst>
 </file>
@@ -539,12 +593,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43E4F913-EFD9-4818-926C-D0A818E637D6}">
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -1093,6 +1149,356 @@
         <v>39</v>
       </c>
     </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>44</v>
+      </c>
+      <c r="B40" t="s">
+        <v>30</v>
+      </c>
+      <c r="C40" t="s">
+        <v>38</v>
+      </c>
+      <c r="D40" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>45</v>
+      </c>
+      <c r="B41" t="s">
+        <v>30</v>
+      </c>
+      <c r="C41" t="s">
+        <v>38</v>
+      </c>
+      <c r="D41" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>46</v>
+      </c>
+      <c r="B42" t="s">
+        <v>30</v>
+      </c>
+      <c r="C42" t="s">
+        <v>38</v>
+      </c>
+      <c r="D42" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>47</v>
+      </c>
+      <c r="B43" t="s">
+        <v>30</v>
+      </c>
+      <c r="C43" t="s">
+        <v>38</v>
+      </c>
+      <c r="D43" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>48</v>
+      </c>
+      <c r="B44" t="s">
+        <v>30</v>
+      </c>
+      <c r="C44" t="s">
+        <v>38</v>
+      </c>
+      <c r="D44" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>44</v>
+      </c>
+      <c r="B45" t="s">
+        <v>30</v>
+      </c>
+      <c r="C45" t="s">
+        <v>38</v>
+      </c>
+      <c r="D45" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>42</v>
+      </c>
+      <c r="B46" t="s">
+        <v>30</v>
+      </c>
+      <c r="C46" t="s">
+        <v>38</v>
+      </c>
+      <c r="D46" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>37</v>
+      </c>
+      <c r="B47" t="s">
+        <v>30</v>
+      </c>
+      <c r="C47" t="s">
+        <v>38</v>
+      </c>
+      <c r="D47" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>49</v>
+      </c>
+      <c r="B48" t="s">
+        <v>30</v>
+      </c>
+      <c r="C48" t="s">
+        <v>38</v>
+      </c>
+      <c r="D48" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>50</v>
+      </c>
+      <c r="B49" t="s">
+        <v>30</v>
+      </c>
+      <c r="C49" t="s">
+        <v>38</v>
+      </c>
+      <c r="D49" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>44</v>
+      </c>
+      <c r="B50" t="s">
+        <v>30</v>
+      </c>
+      <c r="C50" t="s">
+        <v>38</v>
+      </c>
+      <c r="D50" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>51</v>
+      </c>
+      <c r="B51" t="s">
+        <v>30</v>
+      </c>
+      <c r="C51" t="s">
+        <v>38</v>
+      </c>
+      <c r="D51" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>52</v>
+      </c>
+      <c r="B52" t="s">
+        <v>30</v>
+      </c>
+      <c r="C52" t="s">
+        <v>38</v>
+      </c>
+      <c r="D52" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>53</v>
+      </c>
+      <c r="B53" t="s">
+        <v>30</v>
+      </c>
+      <c r="C53" t="s">
+        <v>38</v>
+      </c>
+      <c r="D53" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>54</v>
+      </c>
+      <c r="B54" t="s">
+        <v>30</v>
+      </c>
+      <c r="C54" t="s">
+        <v>38</v>
+      </c>
+      <c r="D54" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>55</v>
+      </c>
+      <c r="B55" t="s">
+        <v>30</v>
+      </c>
+      <c r="C55" t="s">
+        <v>38</v>
+      </c>
+      <c r="D55" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>56</v>
+      </c>
+      <c r="B56" t="s">
+        <v>30</v>
+      </c>
+      <c r="C56" t="s">
+        <v>38</v>
+      </c>
+      <c r="D56" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>57</v>
+      </c>
+      <c r="B57" t="s">
+        <v>30</v>
+      </c>
+      <c r="C57" t="s">
+        <v>38</v>
+      </c>
+      <c r="D57" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>58</v>
+      </c>
+      <c r="B58" t="s">
+        <v>30</v>
+      </c>
+      <c r="C58" t="s">
+        <v>38</v>
+      </c>
+      <c r="D58" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>59</v>
+      </c>
+      <c r="B59" t="s">
+        <v>30</v>
+      </c>
+      <c r="C59" t="s">
+        <v>38</v>
+      </c>
+      <c r="D59" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>60</v>
+      </c>
+      <c r="B60" t="s">
+        <v>30</v>
+      </c>
+      <c r="C60" t="s">
+        <v>38</v>
+      </c>
+      <c r="D60" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>57</v>
+      </c>
+      <c r="B61" t="s">
+        <v>30</v>
+      </c>
+      <c r="C61" t="s">
+        <v>38</v>
+      </c>
+      <c r="D61" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>61</v>
+      </c>
+      <c r="B62" t="s">
+        <v>30</v>
+      </c>
+      <c r="C62" t="s">
+        <v>38</v>
+      </c>
+      <c r="D62" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>55</v>
+      </c>
+      <c r="B63" t="s">
+        <v>30</v>
+      </c>
+      <c r="C63" t="s">
+        <v>38</v>
+      </c>
+      <c r="D63" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>56</v>
+      </c>
+      <c r="B64" t="s">
+        <v>30</v>
+      </c>
+      <c r="C64" t="s">
+        <v>38</v>
+      </c>
+      <c r="D64" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
corrected amplicon data import pipeline
</commit_message>
<xml_diff>
--- a/inst/extdata/makers_details.xlsx
+++ b/inst/extdata/makers_details.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dev\MalReBay-Package\MalReBay\inst\extdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dev\MalReBay-Package\MalReBay_manuscript\Datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{803EF4EC-DABF-4F30-B70D-1C4D56819608}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68742F34-16E4-455A-8A7D-B27CBE827BAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B200665-48F8-48D7-B17C-7D3B5710279D}"/>
   </bookViews>
@@ -36,11 +36,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="64">
   <si>
     <t>marker_id</t>
   </si>
   <si>
+    <t xml:space="preserve">markertype </t>
+  </si>
+  <si>
     <t xml:space="preserve">binning_method </t>
   </si>
   <si>
@@ -125,7 +128,106 @@
     <t>msp_glurp</t>
   </si>
   <si>
+    <t>ampseq</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cpmp </t>
+  </si>
+  <si>
+    <t xml:space="preserve">cpp </t>
+  </si>
+  <si>
+    <t xml:space="preserve">amaD3 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ama1-D3 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">csp </t>
+  </si>
+  <si>
+    <t xml:space="preserve">msp7 </t>
+  </si>
+  <si>
+    <t>csp2</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>exact</t>
+  </si>
+  <si>
     <t>repeatlength</t>
+  </si>
+  <si>
+    <t>SERA2</t>
+  </si>
+  <si>
+    <t>cpp2</t>
+  </si>
+  <si>
+    <t>TRAP3</t>
+  </si>
+  <si>
+    <t>cpmp1</t>
+  </si>
+  <si>
+    <t>celtos</t>
+  </si>
+  <si>
+    <t>surfin1.1</t>
+  </si>
+  <si>
+    <t>ama1-D2</t>
+  </si>
+  <si>
+    <t>ama1-D2.1</t>
+  </si>
+  <si>
+    <t>TRAP2</t>
+  </si>
+  <si>
+    <t>ama1-D3.3</t>
+  </si>
+  <si>
+    <t>csp1</t>
+  </si>
+  <si>
+    <t>msp7.2</t>
+  </si>
+  <si>
+    <t>ama1-D2.3</t>
+  </si>
+  <si>
+    <t>ama1-D3.2</t>
+  </si>
+  <si>
+    <t>cpp3</t>
+  </si>
+  <si>
+    <t>msp7.3</t>
+  </si>
+  <si>
+    <t>cpmp3</t>
+  </si>
+  <si>
+    <t>TRAP4_</t>
+  </si>
+  <si>
+    <t>ama1-D3.4</t>
+  </si>
+  <si>
+    <t>cpmp2</t>
+  </si>
+  <si>
+    <t>cpp1</t>
+  </si>
+  <si>
+    <t>polya</t>
+  </si>
+  <si>
+    <t>D3</t>
   </si>
 </sst>
 </file>
@@ -167,7 +269,18 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -497,335 +610,846 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43E4F913-EFD9-4818-926C-D0A818E637D6}">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:D59"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>313</v>
       </c>
-      <c r="B2">
-        <v>2</v>
-      </c>
-      <c r="C2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>383</v>
       </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4">
         <v>3</v>
       </c>
-      <c r="C4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5">
         <v>3</v>
       </c>
-      <c r="B5">
+      <c r="D5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6">
         <v>3</v>
       </c>
-      <c r="C5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6">
+      <c r="D6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7">
         <v>3</v>
       </c>
-      <c r="C6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7">
+      <c r="D7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8">
         <v>3</v>
       </c>
-      <c r="C7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8">
+      <c r="D8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9">
         <v>2490</v>
       </c>
-      <c r="B8">
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9">
         <v>3</v>
       </c>
-      <c r="C8" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9">
-        <v>3</v>
-      </c>
-      <c r="C9" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>7</v>
       </c>
-      <c r="B10">
-        <v>2</v>
-      </c>
-      <c r="C10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="D10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>8</v>
       </c>
-      <c r="B11">
-        <v>2</v>
-      </c>
-      <c r="C11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
+      </c>
+      <c r="D11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
-      <c r="B12">
-        <v>2</v>
-      </c>
-      <c r="C12" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12">
+        <v>2</v>
+      </c>
+      <c r="D12" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>10</v>
       </c>
-      <c r="B13">
-        <v>2</v>
-      </c>
-      <c r="C13" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13">
+        <v>2</v>
+      </c>
+      <c r="D13" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>11</v>
       </c>
-      <c r="B14">
-        <v>2</v>
-      </c>
-      <c r="C14" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14">
+        <v>2</v>
+      </c>
+      <c r="D14" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>12</v>
       </c>
-      <c r="B15">
-        <v>2</v>
-      </c>
-      <c r="C15" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15">
+        <v>2</v>
+      </c>
+      <c r="D15" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>13</v>
       </c>
-      <c r="B16">
-        <v>2</v>
-      </c>
-      <c r="C16" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16">
+        <v>2</v>
+      </c>
+      <c r="D16" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>14</v>
       </c>
-      <c r="B17">
-        <v>3</v>
-      </c>
-      <c r="C17" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17">
+        <v>2</v>
+      </c>
+      <c r="D17" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>15</v>
       </c>
-      <c r="B18">
+      <c r="B18" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18">
         <v>3</v>
       </c>
-      <c r="C18" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D18" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>16</v>
       </c>
-      <c r="B19">
+      <c r="B19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19">
         <v>3</v>
       </c>
-      <c r="C19" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D19" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>17</v>
       </c>
-      <c r="B20">
+      <c r="B20" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20">
         <v>3</v>
       </c>
-      <c r="C20" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D20" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>18</v>
       </c>
-      <c r="B21">
+      <c r="B21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21">
         <v>3</v>
       </c>
-      <c r="C21" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D21" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>19</v>
       </c>
-      <c r="B22">
-        <v>2</v>
-      </c>
-      <c r="C22" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22">
+        <v>3</v>
+      </c>
+      <c r="D22" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>20</v>
       </c>
-      <c r="B23">
-        <v>2</v>
-      </c>
-      <c r="C23" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B23" t="s">
+        <v>29</v>
+      </c>
+      <c r="C23">
+        <v>2</v>
+      </c>
+      <c r="D23" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>21</v>
       </c>
-      <c r="B24">
-        <v>2</v>
-      </c>
-      <c r="C24" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B24" t="s">
+        <v>29</v>
+      </c>
+      <c r="C24">
+        <v>2</v>
+      </c>
+      <c r="D24" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>22</v>
       </c>
-      <c r="B25">
-        <v>2</v>
-      </c>
-      <c r="C25" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B25" t="s">
+        <v>29</v>
+      </c>
+      <c r="C25">
+        <v>2</v>
+      </c>
+      <c r="D25" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>23</v>
       </c>
-      <c r="B26">
-        <v>2</v>
-      </c>
-      <c r="C26" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B26" t="s">
+        <v>29</v>
+      </c>
+      <c r="C26">
+        <v>2</v>
+      </c>
+      <c r="D26" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>24</v>
       </c>
-      <c r="B27">
-        <v>2</v>
-      </c>
-      <c r="C27" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B27" t="s">
+        <v>29</v>
+      </c>
+      <c r="C27">
+        <v>2</v>
+      </c>
+      <c r="D27" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>25</v>
       </c>
-      <c r="B28">
-        <v>2</v>
-      </c>
-      <c r="C28" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B28" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28">
+        <v>2</v>
+      </c>
+      <c r="D28" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>26</v>
       </c>
-      <c r="B29">
-        <v>2</v>
-      </c>
-      <c r="C29" t="s">
-        <v>28</v>
+      <c r="B29" t="s">
+        <v>29</v>
+      </c>
+      <c r="C29">
+        <v>2</v>
+      </c>
+      <c r="D29" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>27</v>
+      </c>
+      <c r="B30" t="s">
+        <v>29</v>
+      </c>
+      <c r="C30">
+        <v>2</v>
+      </c>
+      <c r="D30" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>31</v>
+      </c>
+      <c r="B31" t="s">
+        <v>30</v>
+      </c>
+      <c r="C31" t="s">
+        <v>38</v>
+      </c>
+      <c r="D31" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>32</v>
+      </c>
+      <c r="B32" t="s">
+        <v>30</v>
+      </c>
+      <c r="C32" t="s">
+        <v>38</v>
+      </c>
+      <c r="D32" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>33</v>
+      </c>
+      <c r="B33" t="s">
+        <v>30</v>
+      </c>
+      <c r="C33" t="s">
+        <v>38</v>
+      </c>
+      <c r="D33" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>34</v>
+      </c>
+      <c r="B34" t="s">
+        <v>30</v>
+      </c>
+      <c r="C34" t="s">
+        <v>38</v>
+      </c>
+      <c r="D34" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>35</v>
+      </c>
+      <c r="B35" t="s">
+        <v>30</v>
+      </c>
+      <c r="C35" t="s">
+        <v>38</v>
+      </c>
+      <c r="D35" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>36</v>
+      </c>
+      <c r="B36" t="s">
+        <v>30</v>
+      </c>
+      <c r="C36" t="s">
+        <v>38</v>
+      </c>
+      <c r="D36" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>41</v>
+      </c>
+      <c r="B37" t="s">
+        <v>30</v>
+      </c>
+      <c r="C37" t="s">
+        <v>38</v>
+      </c>
+      <c r="D37" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>43</v>
+      </c>
+      <c r="B38" t="s">
+        <v>30</v>
+      </c>
+      <c r="C38" t="s">
+        <v>38</v>
+      </c>
+      <c r="D38" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>42</v>
+      </c>
+      <c r="B39" t="s">
+        <v>30</v>
+      </c>
+      <c r="C39" t="s">
+        <v>38</v>
+      </c>
+      <c r="D39" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>37</v>
+      </c>
+      <c r="B40" t="s">
+        <v>30</v>
+      </c>
+      <c r="C40" t="s">
+        <v>38</v>
+      </c>
+      <c r="D40" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>44</v>
+      </c>
+      <c r="B41" t="s">
+        <v>30</v>
+      </c>
+      <c r="C41" t="s">
+        <v>38</v>
+      </c>
+      <c r="D41" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>45</v>
+      </c>
+      <c r="B42" t="s">
+        <v>30</v>
+      </c>
+      <c r="C42" t="s">
+        <v>38</v>
+      </c>
+      <c r="D42" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>46</v>
+      </c>
+      <c r="B43" t="s">
+        <v>30</v>
+      </c>
+      <c r="C43" t="s">
+        <v>38</v>
+      </c>
+      <c r="D43" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>47</v>
+      </c>
+      <c r="B44" t="s">
+        <v>30</v>
+      </c>
+      <c r="C44" t="s">
+        <v>38</v>
+      </c>
+      <c r="D44" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>48</v>
+      </c>
+      <c r="B45" t="s">
+        <v>30</v>
+      </c>
+      <c r="C45" t="s">
+        <v>38</v>
+      </c>
+      <c r="D45" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>49</v>
+      </c>
+      <c r="B46" t="s">
+        <v>30</v>
+      </c>
+      <c r="C46" t="s">
+        <v>38</v>
+      </c>
+      <c r="D46" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>50</v>
+      </c>
+      <c r="B47" t="s">
+        <v>30</v>
+      </c>
+      <c r="C47" t="s">
+        <v>38</v>
+      </c>
+      <c r="D47" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>51</v>
+      </c>
+      <c r="B48" t="s">
+        <v>30</v>
+      </c>
+      <c r="C48" t="s">
+        <v>38</v>
+      </c>
+      <c r="D48" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>52</v>
+      </c>
+      <c r="B49" t="s">
+        <v>30</v>
+      </c>
+      <c r="C49" t="s">
+        <v>38</v>
+      </c>
+      <c r="D49" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>53</v>
+      </c>
+      <c r="B50" t="s">
+        <v>30</v>
+      </c>
+      <c r="C50" t="s">
+        <v>38</v>
+      </c>
+      <c r="D50" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>54</v>
+      </c>
+      <c r="B51" t="s">
+        <v>30</v>
+      </c>
+      <c r="C51" t="s">
+        <v>38</v>
+      </c>
+      <c r="D51" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>55</v>
+      </c>
+      <c r="B52" t="s">
+        <v>30</v>
+      </c>
+      <c r="C52" t="s">
+        <v>38</v>
+      </c>
+      <c r="D52" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>56</v>
+      </c>
+      <c r="B53" t="s">
+        <v>30</v>
+      </c>
+      <c r="C53" t="s">
+        <v>38</v>
+      </c>
+      <c r="D53" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>57</v>
+      </c>
+      <c r="B54" t="s">
+        <v>30</v>
+      </c>
+      <c r="C54" t="s">
+        <v>38</v>
+      </c>
+      <c r="D54" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>58</v>
+      </c>
+      <c r="B55" t="s">
+        <v>30</v>
+      </c>
+      <c r="C55" t="s">
+        <v>38</v>
+      </c>
+      <c r="D55" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>59</v>
+      </c>
+      <c r="B56" t="s">
+        <v>30</v>
+      </c>
+      <c r="C56" t="s">
+        <v>38</v>
+      </c>
+      <c r="D56" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>60</v>
+      </c>
+      <c r="B57" t="s">
+        <v>30</v>
+      </c>
+      <c r="C57" t="s">
+        <v>38</v>
+      </c>
+      <c r="D57" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>61</v>
+      </c>
+      <c r="B58" t="s">
+        <v>30</v>
+      </c>
+      <c r="C58" t="s">
+        <v>38</v>
+      </c>
+      <c r="D58" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>63</v>
+      </c>
+      <c r="B59" t="s">
+        <v>30</v>
+      </c>
+      <c r="C59" t="s">
+        <v>38</v>
+      </c>
+      <c r="D59" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A1:A1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>